<commit_message>
Ledger not working and db download
</commit_message>
<xml_diff>
--- a/data/REPORTING_SHEET_FEB_2026.xlsx
+++ b/data/REPORTING_SHEET_FEB_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oriokie/treasury/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E183F59-121E-A14E-8B1F-CEF32C654797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7060E17F-6780-A84E-BB59-2ACF23F0C106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16060" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16060" tabRatio="500" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OFFERING SUMMARY" sheetId="1" r:id="rId1"/>
@@ -8718,7 +8718,7 @@
     </row>
     <row r="174" spans="2:13" ht="17" x14ac:dyDescent="0.2">
       <c r="B174" s="105" t="s">
-        <v>17</v>
+        <v>138</v>
       </c>
       <c r="C174" s="115">
         <f>L152</f>
@@ -34818,6 +34818,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="8a35f1cb-0131-4512-be3c-ecf28089e959" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010069A88C08EA00054DBAE2359CFE666181" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2f10decbf550d34d8dc59f01efc786">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="8a35f1cb-0131-4512-be3c-ecf28089e959" xmlns:ns4="cf704824-8b6b-4d3c-b7b8-83e18488b4b0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29459a6fc9f1377b70897304ad882a2c" ns3:_="" ns4:_="">
     <xsd:import namespace="8a35f1cb-0131-4512-be3c-ecf28089e959"/>
@@ -35038,24 +35055,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="8a35f1cb-0131-4512-be3c-ecf28089e959" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21F3339F-D757-4C26-B7B6-E947332AF777}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7E5D1D6-7731-41EC-B0F8-B6FD822B49D9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8a35f1cb-0131-4512-be3c-ecf28089e959"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12F3DE46-E566-4693-AF4D-12A6E4E0ABC7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -35072,22 +35090,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7E5D1D6-7731-41EC-B0F8-B6FD822B49D9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="8a35f1cb-0131-4512-be3c-ecf28089e959"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21F3339F-D757-4C26-B7B6-E947332AF777}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>